<commit_message>
🔢 Standardize all tables to 2 decimal places
FORMAT IMPROVEMENT: Consistent decimal formatting across all tables

Changes:
- Updated generate_classification_tables_from_experiment.py
- Changed metrics from 0.0000 (4 decimals) → 0.00 (2 decimals)
- Regenerated all 6 tables with consistent formatting

Results:
✓ Table 1: Dataset Statistics - 2 decimals
✓ Table 2: Detection Performance - 2 decimals
✓ Table 3-6: Classification Performance - 2 decimals

Examples:
- Detection: mAP@50 = 96.02% (not 96.0200%)
- Classification: Accuracy = 0.93 (not 0.9340)
- Per-class: Precision = 0.98, F1 = 0.96 (not 0.9787, 0.9583)

Benefits:
✅ More readable and cleaner
✅ Standard journal format (2 decimals typical)
✅ Consistent across all tables
✅ Less visual clutter

User Request: 'untuk semua tabel buat 2 angka dibelakang koma saja'
</commit_message>
<xml_diff>
--- a/luaran/laporan_akhir/tables/Table3_iml_lifecycle.xlsx
+++ b/luaran/laporan_akhir/tables/Table3_iml_lifecycle.xlsx
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -91,7 +90,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -100,7 +99,7 @@
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>

</xml_diff>